<commit_message>
add shared link and export excel
</commit_message>
<xml_diff>
--- a/docs/examples/reference-case/generated/PM-advanced-7-2D-reference-case-equivalent-block-LC1-theta15.xlsx
+++ b/docs/examples/reference-case/generated/PM-advanced-7-2D-reference-case-equivalent-block-LC1-theta15.xlsx
@@ -87,7 +87,7 @@
     <t>Generated</t>
   </si>
   <si>
-    <t>2026-08-08 01:04:17</t>
+    <t>2026-08-10 06:51:06</t>
   </si>
   <si>
     <t>Calculation profile</t>
@@ -58178,7 +58178,7 @@
         <v>-2085.2180703321987</v>
       </c>
       <c r="G7" s="18">
-        <v>-803.8345866297666</v>
+        <v>-803.8345866297667</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
@@ -58198,7 +58198,7 @@
         <v>-1841.734820783854</v>
       </c>
       <c r="G8" s="18">
-        <v>-709.9737765607335</v>
+        <v>-709.9737765607338</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
@@ -58215,10 +58215,10 @@
         <v>-1844.655676882907</v>
       </c>
       <c r="F9" s="18">
-        <v>-1721.195317179876</v>
+        <v>-1721.1953171798762</v>
       </c>
       <c r="G9" s="18">
-        <v>-663.5067794487125</v>
+        <v>-663.5067794487127</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
@@ -58232,13 +58232,13 @@
         <v>17670.345615483235</v>
       </c>
       <c r="E10" s="18">
-        <v>-1754.204129536191</v>
+        <v>-1754.2041295361912</v>
       </c>
       <c r="F10" s="18">
-        <v>-1636.797572020239</v>
+        <v>-1636.7975720202392</v>
       </c>
       <c r="G10" s="18">
-        <v>-630.9721359224009</v>
+        <v>-630.972135922401</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
@@ -58252,13 +58252,13 @@
         <v>17670.345615483235</v>
       </c>
       <c r="E11" s="18">
-        <v>-1560.2825802294083</v>
+        <v>-1560.2825802294085</v>
       </c>
       <c r="F11" s="18">
         <v>-1455.854935001326</v>
       </c>
       <c r="G11" s="18">
-        <v>-561.2202227286763</v>
+        <v>-561.2202227286764</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
@@ -58272,13 +58272,13 @@
         <v>17670.345615483235</v>
       </c>
       <c r="E12" s="18">
-        <v>-1410.903000692412</v>
+        <v>-1410.9030006924122</v>
       </c>
       <c r="F12" s="18">
-        <v>-1316.4731327476702</v>
+        <v>-1316.4731327476704</v>
       </c>
       <c r="G12" s="18">
-        <v>-507.4896729159985</v>
+        <v>-507.4896729159987</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
@@ -58298,7 +58298,7 @@
         <v>-1198.6665831354362</v>
       </c>
       <c r="G13" s="18">
-        <v>-462.0762073139367</v>
+        <v>-462.07620731393695</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
@@ -58392,13 +58392,13 @@
         <v>17670.345615483235</v>
       </c>
       <c r="E18" s="18">
-        <v>-668.00223294975</v>
+        <v>-668.0022329497502</v>
       </c>
       <c r="F18" s="18">
-        <v>-623.2937288121299</v>
+        <v>-623.29372881213</v>
       </c>
       <c r="G18" s="18">
-        <v>-240.27465710998987</v>
+        <v>-240.27465710999013</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.25">
@@ -58432,13 +58432,13 @@
         <v>17670.345615483235</v>
       </c>
       <c r="E20" s="18">
-        <v>-438.7297266640511</v>
+        <v>-438.7297266640513</v>
       </c>
       <c r="F20" s="18">
-        <v>-409.3661275137289</v>
+        <v>-409.36612751372894</v>
       </c>
       <c r="G20" s="18">
-        <v>-157.8073087760086</v>
+        <v>-157.80730877600908</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.25">
@@ -58492,7 +58492,7 @@
         <v>17670.345615483235</v>
       </c>
       <c r="E23" s="18">
-        <v>-107.13613533782987</v>
+        <v>-107.13613533782988</v>
       </c>
       <c r="F23" s="18">
         <v>-99.96565578884862</v>
@@ -58512,7 +58512,7 @@
         <v>17670.345615483235</v>
       </c>
       <c r="E24" s="18">
-        <v>6.306245291983856e-14</v>
+        <v>6.306245291983853e-14</v>
       </c>
       <c r="F24" s="18">
         <v>2.5140272845185274e-13</v>
@@ -58712,7 +58712,7 @@
         <v>17670.345615483235</v>
       </c>
       <c r="E34" s="18">
-        <v>727.8782030248739</v>
+        <v>727.878203024874</v>
       </c>
       <c r="F34" s="18">
         <v>679.1622795646762</v>
@@ -58795,10 +58795,10 @@
         <v>1024.8358593431167</v>
       </c>
       <c r="F38" s="18">
-        <v>956.244953508121</v>
+        <v>956.2449535081208</v>
       </c>
       <c r="G38" s="18">
-        <v>368.62464307991695</v>
+        <v>368.6246430799174</v>
       </c>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.25">
@@ -58812,13 +58812,13 @@
         <v>17670.345615483235</v>
       </c>
       <c r="E39" s="18">
-        <v>1126.8378543287808</v>
+        <v>1126.837854328781</v>
       </c>
       <c r="F39" s="18">
         <v>1051.4200901542185</v>
       </c>
       <c r="G39" s="18">
-        <v>405.3138832662735</v>
+        <v>405.31388326627325</v>
       </c>
     </row>
     <row r="40" spans="2:7" x14ac:dyDescent="0.25">
@@ -58838,7 +58838,7 @@
         <v>1114.7017796809387</v>
       </c>
       <c r="G40" s="18">
-        <v>429.7084592896051</v>
+        <v>429.7084592896054</v>
       </c>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.25">
@@ -58858,7 +58858,7 @@
         <v>1206.1007065566903</v>
       </c>
       <c r="G41" s="18">
-        <v>464.94200135835837</v>
+        <v>464.9420013583586</v>
       </c>
     </row>
     <row r="42" spans="2:7" x14ac:dyDescent="0.25">
@@ -58918,7 +58918,7 @@
         <v>1667.155385069757</v>
       </c>
       <c r="G44" s="18">
-        <v>642.6748256558326</v>
+        <v>642.6748256558328</v>
       </c>
     </row>
     <row r="45" spans="2:7" x14ac:dyDescent="0.25">
@@ -58938,7 +58938,7 @@
         <v>1763.7063618633147</v>
       </c>
       <c r="G45" s="18">
-        <v>679.8944410158632</v>
+        <v>679.8944410158633</v>
       </c>
     </row>
     <row r="46" spans="2:7" x14ac:dyDescent="0.25">
@@ -58958,7 +58958,7 @@
         <v>2035.9462751534231</v>
       </c>
       <c r="G46" s="18">
-        <v>784.840710798004</v>
+        <v>784.8407107980041</v>
       </c>
     </row>
     <row r="47" spans="2:7" x14ac:dyDescent="0.25">
@@ -58972,13 +58972,13 @@
         <v>17670.345615483235</v>
       </c>
       <c r="E47" s="18">
-        <v>2204.8401184591453</v>
+        <v>2204.8401184591457</v>
       </c>
       <c r="F47" s="18">
         <v>2057.273091439436</v>
       </c>
       <c r="G47" s="18">
-        <v>793.0620248165734</v>
+        <v>793.0620248165735</v>
       </c>
     </row>
     <row r="48" spans="2:7" x14ac:dyDescent="0.25">
@@ -59018,7 +59018,7 @@
         <v>2245.8117257945933</v>
       </c>
       <c r="G49" s="18">
-        <v>865.7421331308439</v>
+        <v>865.742133130844</v>
       </c>
     </row>
     <row r="50" spans="2:7" x14ac:dyDescent="0.25">
@@ -59029,7 +59029,7 @@
         <v>1</v>
       </c>
       <c r="D50" s="18">
-        <v>16864.238544529213</v>
+        <v>16864.238544529217</v>
       </c>
       <c r="E50" s="18">
         <v>2561.8928736680623</v>
@@ -59038,7 +59038,7 @@
         <v>2390.428778949767</v>
       </c>
       <c r="G50" s="18">
-        <v>921.4908295365319</v>
+        <v>921.490829536532</v>
       </c>
     </row>
     <row r="51" spans="2:7" x14ac:dyDescent="0.25">
@@ -59058,7 +59058,7 @@
         <v>2455.286050549801</v>
       </c>
       <c r="G51" s="18">
-        <v>946.4927796194994</v>
+        <v>946.4927796194996</v>
       </c>
     </row>
     <row r="52" spans="2:7" x14ac:dyDescent="0.25">
@@ -59078,7 +59078,7 @@
         <v>2706.9912369924655</v>
       </c>
       <c r="G52" s="18">
-        <v>1043.523079411825</v>
+        <v>1043.5230794118252</v>
       </c>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.25">
@@ -59089,7 +59089,7 @@
         <v>1</v>
       </c>
       <c r="D53" s="18">
-        <v>15276.558196044114</v>
+        <v>15276.558196044116</v>
       </c>
       <c r="E53" s="18">
         <v>3097.997644831612</v>
@@ -59098,7 +59098,7 @@
         <v>2890.6527682872984</v>
       </c>
       <c r="G53" s="18">
-        <v>1114.3231042095442</v>
+        <v>1114.3231042095445</v>
       </c>
     </row>
     <row r="54" spans="2:7" x14ac:dyDescent="0.25">
@@ -59112,7 +59112,7 @@
         <v>13681.717876580104</v>
       </c>
       <c r="E54" s="18">
-        <v>3596.929416293759</v>
+        <v>3596.9294162937595</v>
       </c>
       <c r="F54" s="18">
         <v>3356.1916975274885</v>
@@ -59138,7 +59138,7 @@
         <v>3375.1032904019935</v>
       </c>
       <c r="G55" s="18">
-        <v>1301.0748357081118</v>
+        <v>1301.074835708112</v>
       </c>
     </row>
     <row r="56" spans="2:7" x14ac:dyDescent="0.25">
@@ -59158,7 +59158,7 @@
         <v>3555.6411961049726</v>
       </c>
       <c r="G56" s="18">
-        <v>1370.6707282751847</v>
+        <v>1370.670728275185</v>
       </c>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.25">
@@ -59178,7 +59178,7 @@
         <v>3562.93012622371</v>
       </c>
       <c r="G57" s="18">
-        <v>1373.4805514837642</v>
+        <v>1373.4805514837644</v>
       </c>
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.25">
@@ -59189,16 +59189,16 @@
         <v>1</v>
       </c>
       <c r="D58" s="18">
-        <v>11877.474664358297</v>
+        <v>11877.474664358302</v>
       </c>
       <c r="E58" s="18">
-        <v>3971.272503787441</v>
+        <v>3971.27250378744</v>
       </c>
       <c r="F58" s="18">
-        <v>3705.4804982979113</v>
+        <v>3705.4804982979103</v>
       </c>
       <c r="G58" s="18">
-        <v>1428.4325591612778</v>
+        <v>1428.4325591612776</v>
       </c>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.25">
@@ -59218,7 +59218,7 @@
         <v>3706.195987401732</v>
       </c>
       <c r="G59" s="18">
-        <v>1428.7083743847263</v>
+        <v>1428.7083743847265</v>
       </c>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.25">
@@ -59232,13 +59232,13 @@
         <v>11872.94275686741</v>
       </c>
       <c r="E60" s="18">
-        <v>3972.086613366593</v>
+        <v>3972.0866133665936</v>
       </c>
       <c r="F60" s="18">
         <v>3706.240120601883</v>
       </c>
       <c r="G60" s="18">
-        <v>1428.7253873740171</v>
+        <v>1428.7253873740178</v>
       </c>
     </row>
     <row r="61" spans="2:7" x14ac:dyDescent="0.25">
@@ -59258,7 +59258,7 @@
         <v>3815.372046731526</v>
       </c>
       <c r="G61" s="18">
-        <v>1470.7948562591378</v>
+        <v>1470.7948562591382</v>
       </c>
     </row>
     <row r="62" spans="2:7" x14ac:dyDescent="0.25">
@@ -59298,7 +59298,7 @@
         <v>3902.016274038258</v>
       </c>
       <c r="G63" s="18">
-        <v>1504.1955003605326</v>
+        <v>1504.1955003605328</v>
       </c>
     </row>
     <row r="64" spans="2:7" x14ac:dyDescent="0.25">
@@ -59312,13 +59312,13 @@
         <v>10331.547199996237</v>
       </c>
       <c r="E64" s="18">
-        <v>4182.594711509763</v>
+        <v>4182.594711509764</v>
       </c>
       <c r="F64" s="18">
         <v>3902.659190725974</v>
       </c>
       <c r="G64" s="18">
-        <v>1504.4433395085143</v>
+        <v>1504.4433395085146</v>
       </c>
     </row>
     <row r="65" spans="2:7" x14ac:dyDescent="0.25">
@@ -59329,16 +59329,16 @@
         <v>1</v>
       </c>
       <c r="D65" s="18">
-        <v>9735.550746902774</v>
+        <v>9735.550746902754</v>
       </c>
       <c r="E65" s="18">
-        <v>4243.095112882572</v>
+        <v>4243.095112882574</v>
       </c>
       <c r="F65" s="18">
-        <v>3959.1103804170193</v>
+        <v>3959.110380417021</v>
       </c>
       <c r="G65" s="18">
-        <v>1526.204813464488</v>
+        <v>1526.204813464489</v>
       </c>
     </row>
     <row r="66" spans="2:7" x14ac:dyDescent="0.25">
@@ -59378,7 +59378,7 @@
         <v>3968.8619479295567</v>
       </c>
       <c r="G67" s="18">
-        <v>1529.9639633356494</v>
+        <v>1529.9639633356496</v>
       </c>
     </row>
     <row r="68" spans="2:7" x14ac:dyDescent="0.25">
@@ -59392,13 +59392,13 @@
         <v>8989.491340964054</v>
       </c>
       <c r="E68" s="18">
-        <v>4309.4391925400305</v>
+        <v>4309.439192540031</v>
       </c>
       <c r="F68" s="18">
         <v>4021.0141387498406</v>
       </c>
       <c r="G68" s="18">
-        <v>1550.06820823277</v>
+        <v>1550.0682082327703</v>
       </c>
     </row>
     <row r="69" spans="2:7" x14ac:dyDescent="0.25">
@@ -59418,7 +59418,7 @@
         <v>4022.32838617423</v>
       </c>
       <c r="G69" s="18">
-        <v>1550.5748399132374</v>
+        <v>1550.5748399132376</v>
       </c>
     </row>
     <row r="70" spans="2:7" x14ac:dyDescent="0.25">
@@ -59435,10 +59435,10 @@
         <v>4564.181888541133</v>
       </c>
       <c r="F70" s="18">
-        <v>4258.70724372203</v>
+        <v>4258.7072437220295</v>
       </c>
       <c r="G70" s="18">
-        <v>1641.6969647156</v>
+        <v>1641.6969647156002</v>
       </c>
     </row>
     <row r="71" spans="2:7" x14ac:dyDescent="0.25">
@@ -59455,10 +59455,10 @@
         <v>4572.128443314535</v>
       </c>
       <c r="F71" s="18">
-        <v>4266.121946116141</v>
+        <v>4266.12194611614</v>
       </c>
       <c r="G71" s="18">
-        <v>1644.555272112199</v>
+        <v>1644.5552721121994</v>
       </c>
     </row>
     <row r="72" spans="2:7" x14ac:dyDescent="0.25">
@@ -59478,7 +59478,7 @@
         <v>4409.107124733829</v>
       </c>
       <c r="G72" s="18">
-        <v>1699.6748941716905</v>
+        <v>1699.6748941716908</v>
       </c>
     </row>
     <row r="73" spans="2:7" x14ac:dyDescent="0.25">
@@ -59492,13 +59492,13 @@
         <v>7663.159543900818</v>
       </c>
       <c r="E73" s="18">
-        <v>4737.863497598904</v>
+        <v>4737.863497598905</v>
       </c>
       <c r="F73" s="18">
         <v>4420.764572868492</v>
       </c>
       <c r="G73" s="18">
-        <v>1704.1687455035049</v>
+        <v>1704.168745503505</v>
       </c>
     </row>
     <row r="74" spans="2:7" x14ac:dyDescent="0.25">
@@ -59518,7 +59518,7 @@
         <v>4514.62672363901</v>
       </c>
       <c r="G74" s="18">
-        <v>1740.3518403261867</v>
+        <v>1740.3518403261871</v>
       </c>
     </row>
     <row r="75" spans="2:7" x14ac:dyDescent="0.25">
@@ -59538,7 +59538,7 @@
         <v>4532.64997006488</v>
       </c>
       <c r="G75" s="18">
-        <v>1747.2996550639314</v>
+        <v>1747.2996550639316</v>
       </c>
     </row>
     <row r="76" spans="2:7" x14ac:dyDescent="0.25">
@@ -59558,7 +59558,7 @@
         <v>4584.03156912068</v>
       </c>
       <c r="G76" s="18">
-        <v>1767.1068431106066</v>
+        <v>1767.106843110607</v>
       </c>
     </row>
     <row r="77" spans="2:7" x14ac:dyDescent="0.25">
@@ -59578,7 +59578,7 @@
         <v>4619.717379350748</v>
       </c>
       <c r="G77" s="18">
-        <v>1780.8634323724027</v>
+        <v>1780.863432372403</v>
       </c>
     </row>
     <row r="78" spans="2:7" x14ac:dyDescent="0.25">
@@ -59615,10 +59615,10 @@
         <v>4893.415175265811</v>
       </c>
       <c r="F79" s="18">
-        <v>4565.9053829042</v>
+        <v>4565.9053829041995</v>
       </c>
       <c r="G79" s="18">
-        <v>1760.1193459217982</v>
+        <v>1760.1193459217986</v>
       </c>
     </row>
     <row r="80" spans="2:7" x14ac:dyDescent="0.25">
@@ -59629,16 +59629,16 @@
         <v>1</v>
       </c>
       <c r="D80" s="18">
-        <v>4822.094624327781</v>
+        <v>4822.09462432778</v>
       </c>
       <c r="E80" s="18">
-        <v>4668.85725985605</v>
+        <v>4668.8572598560495</v>
       </c>
       <c r="F80" s="18">
-        <v>4356.376831162731</v>
+        <v>4356.37683116273</v>
       </c>
       <c r="G80" s="18">
-        <v>1679.3477953714976</v>
+        <v>1679.347795371498</v>
       </c>
     </row>
     <row r="81" spans="2:7" x14ac:dyDescent="0.25">
@@ -59669,16 +59669,16 @@
         <v>1</v>
       </c>
       <c r="D82" s="18">
-        <v>3176.7687287078643</v>
+        <v>3176.768728707864</v>
       </c>
       <c r="E82" s="18">
         <v>4105.836644579057</v>
       </c>
       <c r="F82" s="18">
-        <v>3831.0384394862845</v>
+        <v>3831.038439486284</v>
       </c>
       <c r="G82" s="18">
-        <v>1476.8341230980225</v>
+        <v>1476.834123098023</v>
       </c>
     </row>
     <row r="83" spans="2:7" x14ac:dyDescent="0.25">
@@ -59698,7 +59698,7 @@
         <v>3520.00556497416</v>
       </c>
       <c r="G83" s="18">
-        <v>1356.933482647554</v>
+        <v>1356.9334826475542</v>
       </c>
     </row>
     <row r="84" spans="2:7" x14ac:dyDescent="0.25">
@@ -59709,13 +59709,13 @@
         <v>1</v>
       </c>
       <c r="D84" s="18">
-        <v>2023.0816349536217</v>
+        <v>2023.0816349536212</v>
       </c>
       <c r="E84" s="18">
-        <v>3662.6933932567604</v>
+        <v>3662.69339325676</v>
       </c>
       <c r="F84" s="18">
-        <v>3417.554178670374</v>
+        <v>3417.5541786703734</v>
       </c>
       <c r="G84" s="18">
         <v>1317.4393074670986</v>
@@ -59729,16 +59729,16 @@
         <v>1</v>
       </c>
       <c r="D85" s="18">
-        <v>-34.313420754170046</v>
+        <v>-34.31342075417191</v>
       </c>
       <c r="E85" s="18">
-        <v>2703.983547010343</v>
+        <v>2703.9835470103426</v>
       </c>
       <c r="F85" s="18">
-        <v>2523.00951184022</v>
+        <v>2523.0095118402196</v>
       </c>
       <c r="G85" s="18">
-        <v>972.599622489343</v>
+        <v>972.5996224893429</v>
       </c>
     </row>
     <row r="86" spans="2:7" x14ac:dyDescent="0.25">
@@ -59749,16 +59749,16 @@
         <v>1</v>
       </c>
       <c r="D86" s="18">
-        <v>-144.58702319349496</v>
+        <v>-144.58702319349518</v>
       </c>
       <c r="E86" s="18">
-        <v>2651.364380401322</v>
+        <v>2651.3643804013213</v>
       </c>
       <c r="F86" s="18">
-        <v>2473.9120763153437</v>
+        <v>2473.9120763153433</v>
       </c>
       <c r="G86" s="18">
-        <v>953.6729608843852</v>
+        <v>953.6729608843854</v>
       </c>
     </row>
     <row r="87" spans="2:7" x14ac:dyDescent="0.25">
@@ -59769,7 +59769,7 @@
         <v>1</v>
       </c>
       <c r="D87" s="18">
-        <v>-152.46417959881057</v>
+        <v>-152.46417959881072</v>
       </c>
       <c r="E87" s="18">
         <v>2647.8458649281206</v>
@@ -59778,7 +59778,7 @@
         <v>2470.6290504196204</v>
       </c>
       <c r="G87" s="18">
-        <v>952.4073811345594</v>
+        <v>952.4073811345595</v>
       </c>
     </row>
     <row r="88" spans="2:7" x14ac:dyDescent="0.25">
@@ -59789,7 +59789,7 @@
         <v>1</v>
       </c>
       <c r="D88" s="18">
-        <v>-1572.5000854716902</v>
+        <v>-1572.5000854716905</v>
       </c>
       <c r="E88" s="18">
         <v>1910.1560306103713</v>
@@ -59798,7 +59798,7 @@
         <v>1782.3118190409944</v>
       </c>
       <c r="G88" s="18">
-        <v>687.0666932576133</v>
+        <v>687.0666932576135</v>
       </c>
     </row>
     <row r="89" spans="2:7" x14ac:dyDescent="0.25">
@@ -59818,7 +59818,7 @@
         <v>1721.0347598272929</v>
       </c>
       <c r="G89" s="18">
-        <v>663.4448858966756</v>
+        <v>663.4448858966757</v>
       </c>
     </row>
     <row r="90" spans="2:7" x14ac:dyDescent="0.25">
@@ -59832,13 +59832,13 @@
         <v>-3589.3994585750506</v>
       </c>
       <c r="E90" s="18">
-        <v>783.8980408469944</v>
+        <v>783.8980408469943</v>
       </c>
       <c r="F90" s="18">
-        <v>731.432783885321</v>
+        <v>731.4327838853209</v>
       </c>
       <c r="G90" s="18">
-        <v>281.96138228758457</v>
+        <v>281.9613822875846</v>
       </c>
     </row>
     <row r="91" spans="2:7" x14ac:dyDescent="0.25">
@@ -59852,7 +59852,7 @@
         <v>-4921.996042232201</v>
       </c>
       <c r="E91" s="18">
-        <v>1.8223386311120322e-14</v>
+        <v>1.8223386311120326e-14</v>
       </c>
       <c r="F91" s="18">
         <v>0</v>
@@ -59872,13 +59872,13 @@
         <v>-3589.39945857505</v>
       </c>
       <c r="E92" s="18">
-        <v>-783.8980408469947</v>
+        <v>-783.8980408469946</v>
       </c>
       <c r="F92" s="18">
-        <v>-731.4327838853213</v>
+        <v>-731.4327838853212</v>
       </c>
       <c r="G92" s="18">
-        <v>-281.9613822875847</v>
+        <v>-281.96138228758474</v>
       </c>
     </row>
     <row r="93" spans="2:7" x14ac:dyDescent="0.25">
@@ -59898,7 +59898,7 @@
         <v>-1721.0347598272929</v>
       </c>
       <c r="G93" s="18">
-        <v>-663.4448858966756</v>
+        <v>-663.4448858966757</v>
       </c>
     </row>
     <row r="94" spans="2:7" x14ac:dyDescent="0.25">
@@ -59909,16 +59909,16 @@
         <v>1</v>
       </c>
       <c r="D94" s="18">
-        <v>-1572.5000854716902</v>
+        <v>-1572.5000854716907</v>
       </c>
       <c r="E94" s="18">
-        <v>-1910.156030610371</v>
+        <v>-1910.1560306103709</v>
       </c>
       <c r="F94" s="18">
-        <v>-1782.3118190409941</v>
+        <v>-1782.311819040994</v>
       </c>
       <c r="G94" s="18">
-        <v>-687.0666932576133</v>
+        <v>-687.0666932576135</v>
       </c>
     </row>
     <row r="95" spans="2:7" x14ac:dyDescent="0.25">
@@ -59929,16 +59929,16 @@
         <v>1</v>
       </c>
       <c r="D95" s="18">
-        <v>-152.46417959880716</v>
+        <v>-152.4641795988073</v>
       </c>
       <c r="E95" s="18">
-        <v>-2647.8458649281224</v>
+        <v>-2647.845864928123</v>
       </c>
       <c r="F95" s="18">
         <v>-2470.6290504196227</v>
       </c>
       <c r="G95" s="18">
-        <v>-952.4073811345603</v>
+        <v>-952.4073811345604</v>
       </c>
     </row>
     <row r="96" spans="2:7" x14ac:dyDescent="0.25">
@@ -59949,7 +59949,7 @@
         <v>1</v>
       </c>
       <c r="D96" s="18">
-        <v>-144.58702319349214</v>
+        <v>-144.58702319349234</v>
       </c>
       <c r="E96" s="18">
         <v>-2651.364380401324</v>
@@ -59958,7 +59958,7 @@
         <v>-2473.912076315346</v>
       </c>
       <c r="G96" s="18">
-        <v>-953.672960884386</v>
+        <v>-953.6729608843862</v>
       </c>
     </row>
     <row r="97" spans="2:7" x14ac:dyDescent="0.25">
@@ -59969,16 +59969,16 @@
         <v>1</v>
       </c>
       <c r="D97" s="18">
-        <v>-34.3134207541761</v>
+        <v>-34.31342075417749</v>
       </c>
       <c r="E97" s="18">
-        <v>-2703.9835470103417</v>
+        <v>-2703.983547010341</v>
       </c>
       <c r="F97" s="18">
-        <v>-2523.0095118402182</v>
+        <v>-2523.009511840218</v>
       </c>
       <c r="G97" s="18">
-        <v>-972.5996224893423</v>
+        <v>-972.5996224893422</v>
       </c>
     </row>
     <row r="98" spans="2:7" x14ac:dyDescent="0.25">
@@ -60029,7 +60029,7 @@
         <v>1</v>
       </c>
       <c r="D100" s="18">
-        <v>3176.7687287078675</v>
+        <v>3176.768728707867</v>
       </c>
       <c r="E100" s="18">
         <v>-4105.836644579058</v>
@@ -60038,7 +60038,7 @@
         <v>-3831.0384394862854</v>
       </c>
       <c r="G100" s="18">
-        <v>-1476.834123098023</v>
+        <v>-1476.8341230980234</v>
       </c>
     </row>
     <row r="101" spans="2:7" x14ac:dyDescent="0.25">
@@ -60058,7 +60058,7 @@
         <v>-4084.766610487395</v>
       </c>
       <c r="G101" s="18">
-        <v>-1574.6442669649002</v>
+        <v>-1574.6442669649005</v>
       </c>
     </row>
     <row r="102" spans="2:7" x14ac:dyDescent="0.25">
@@ -60072,13 +60072,13 @@
         <v>4822.09462432778</v>
       </c>
       <c r="E102" s="18">
-        <v>-4668.85725985605</v>
+        <v>-4668.8572598560495</v>
       </c>
       <c r="F102" s="18">
-        <v>-4356.376831162731</v>
+        <v>-4356.37683116273</v>
       </c>
       <c r="G102" s="18">
-        <v>-1679.3477953714976</v>
+        <v>-1679.3477953714978</v>
       </c>
     </row>
     <row r="103" spans="2:7" x14ac:dyDescent="0.25">
@@ -60098,7 +60098,7 @@
         <v>-4565.905382904201</v>
       </c>
       <c r="G103" s="18">
-        <v>-1760.1193459217989</v>
+        <v>-1760.119345921799</v>
       </c>
     </row>
     <row r="104" spans="2:7" x14ac:dyDescent="0.25">
@@ -60118,7 +60118,7 @@
         <v>-4653.666603488859</v>
       </c>
       <c r="G104" s="18">
-        <v>-1793.9505818363973</v>
+        <v>-1793.9505818363978</v>
       </c>
     </row>
     <row r="105" spans="2:7" x14ac:dyDescent="0.25">
@@ -60138,7 +60138,7 @@
         <v>-4619.717379350747</v>
       </c>
       <c r="G105" s="18">
-        <v>-1780.8634323724025</v>
+        <v>-1780.8634323724027</v>
       </c>
     </row>
     <row r="106" spans="2:7" x14ac:dyDescent="0.25">
@@ -60178,7 +60178,7 @@
         <v>-4532.64997006488</v>
       </c>
       <c r="G107" s="18">
-        <v>-1747.2996550639316</v>
+        <v>-1747.299655063932</v>
       </c>
     </row>
     <row r="108" spans="2:7" x14ac:dyDescent="0.25">
@@ -60198,7 +60198,7 @@
         <v>-4514.62672363901</v>
       </c>
       <c r="G108" s="18">
-        <v>-1740.3518403261871</v>
+        <v>-1740.3518403261874</v>
       </c>
     </row>
     <row r="109" spans="2:7" x14ac:dyDescent="0.25">
@@ -60212,13 +60212,13 @@
         <v>7663.1595439008215</v>
       </c>
       <c r="E109" s="18">
-        <v>-4737.863497598904</v>
+        <v>-4737.863497598905</v>
       </c>
       <c r="F109" s="18">
         <v>-4420.764572868492</v>
       </c>
       <c r="G109" s="18">
-        <v>-1704.1687455035046</v>
+        <v>-1704.1687455035049</v>
       </c>
     </row>
     <row r="110" spans="2:7" x14ac:dyDescent="0.25">
@@ -60238,7 +60238,7 @@
         <v>-4409.107124733828</v>
       </c>
       <c r="G110" s="18">
-        <v>-1699.6748941716903</v>
+        <v>-1699.6748941716905</v>
       </c>
     </row>
     <row r="111" spans="2:7" x14ac:dyDescent="0.25">
@@ -60258,7 +60258,7 @@
         <v>-4266.121946116141</v>
       </c>
       <c r="G111" s="18">
-        <v>-1644.5552721121994</v>
+        <v>-1644.5552721121996</v>
       </c>
     </row>
     <row r="112" spans="2:7" x14ac:dyDescent="0.25">
@@ -60278,7 +60278,7 @@
         <v>-4258.70724372203</v>
       </c>
       <c r="G112" s="18">
-        <v>-1641.6969647156002</v>
+        <v>-1641.6969647156004</v>
       </c>
     </row>
     <row r="113" spans="2:7" x14ac:dyDescent="0.25">
@@ -60338,7 +60338,7 @@
         <v>-3968.8619479295567</v>
       </c>
       <c r="G115" s="18">
-        <v>-1529.9639633356496</v>
+        <v>-1529.96396333565</v>
       </c>
     </row>
     <row r="116" spans="2:7" x14ac:dyDescent="0.25">
@@ -60358,7 +60358,7 @@
         <v>-3968.7743669381002</v>
       </c>
       <c r="G116" s="18">
-        <v>-1529.9302015765963</v>
+        <v>-1529.9302015765966</v>
       </c>
     </row>
     <row r="117" spans="2:7" x14ac:dyDescent="0.25">
@@ -60369,16 +60369,16 @@
         <v>1</v>
       </c>
       <c r="D117" s="18">
-        <v>9735.550746902632</v>
+        <v>9735.550746902609</v>
       </c>
       <c r="E117" s="18">
-        <v>-4243.095112882586</v>
+        <v>-4243.095112882588</v>
       </c>
       <c r="F117" s="18">
-        <v>-3959.1103804170325</v>
+        <v>-3959.110380417035</v>
       </c>
       <c r="G117" s="18">
-        <v>-1526.2048134644933</v>
+        <v>-1526.2048134644942</v>
       </c>
     </row>
     <row r="118" spans="2:7" x14ac:dyDescent="0.25">
@@ -60398,7 +60398,7 @@
         <v>-3902.659190725973</v>
       </c>
       <c r="G118" s="18">
-        <v>-1504.443339508514</v>
+        <v>-1504.4433395085143</v>
       </c>
     </row>
     <row r="119" spans="2:7" x14ac:dyDescent="0.25">
@@ -60415,7 +60415,7 @@
         <v>-4181.905678774245</v>
       </c>
       <c r="F119" s="18">
-        <v>-3902.016274038257</v>
+        <v>-3902.0162740382566</v>
       </c>
       <c r="G119" s="18">
         <v>-1504.1955003605324</v>
@@ -60432,13 +60432,13 @@
         <v>11068.384197665373</v>
       </c>
       <c r="E120" s="18">
-        <v>-4091.26642443663</v>
+        <v>-4091.2664244366306</v>
       </c>
       <c r="F120" s="18">
         <v>-3817.443384867852</v>
       </c>
       <c r="G120" s="18">
-        <v>-1471.5933402442292</v>
+        <v>-1471.5933402442295</v>
       </c>
     </row>
     <row r="121" spans="2:7" x14ac:dyDescent="0.25">
@@ -60449,7 +60449,7 @@
         <v>1</v>
       </c>
       <c r="D121" s="18">
-        <v>11084.131683012323</v>
+        <v>11084.131683012325</v>
       </c>
       <c r="E121" s="18">
         <v>-4089.0465103956262</v>
@@ -60472,13 +60472,13 @@
         <v>11872.942756867404</v>
       </c>
       <c r="E122" s="18">
-        <v>-3972.0866133665945</v>
+        <v>-3972.086613366595</v>
       </c>
       <c r="F122" s="18">
         <v>-3706.240120601884</v>
       </c>
       <c r="G122" s="18">
-        <v>-1428.7253873740174</v>
+        <v>-1428.7253873740178</v>
       </c>
     </row>
     <row r="123" spans="2:7" x14ac:dyDescent="0.25">
@@ -60489,7 +60489,7 @@
         <v>1</v>
       </c>
       <c r="D123" s="18">
-        <v>11873.208198962659</v>
+        <v>11873.20819896266</v>
       </c>
       <c r="E123" s="18">
         <v>-3972.0393145171347</v>
@@ -60509,16 +60509,16 @@
         <v>1</v>
       </c>
       <c r="D124" s="18">
-        <v>11877.474664358317</v>
+        <v>11877.474664358322</v>
       </c>
       <c r="E124" s="18">
-        <v>-3971.272503787438</v>
+        <v>-3971.2725037874375</v>
       </c>
       <c r="F124" s="18">
-        <v>-3705.4804982979085</v>
+        <v>-3705.480498297907</v>
       </c>
       <c r="G124" s="18">
-        <v>-1428.4325591612762</v>
+        <v>-1428.432559161276</v>
       </c>
     </row>
     <row r="125" spans="2:7" x14ac:dyDescent="0.25">
@@ -60535,10 +60535,10 @@
         <v>-3818.4970747215016</v>
       </c>
       <c r="F125" s="18">
-        <v>-3562.930126223712</v>
+        <v>-3562.9301262237113</v>
       </c>
       <c r="G125" s="18">
-        <v>-1373.4805514837647</v>
+        <v>-1373.4805514837649</v>
       </c>
     </row>
     <row r="126" spans="2:7" x14ac:dyDescent="0.25">
@@ -60555,10 +60555,10 @@
         <v>-3810.685313797144</v>
       </c>
       <c r="F126" s="18">
-        <v>-3555.6411961049744</v>
+        <v>-3555.641196104974</v>
       </c>
       <c r="G126" s="18">
-        <v>-1370.6707282751852</v>
+        <v>-1370.6707282751854</v>
       </c>
     </row>
     <row r="127" spans="2:7" x14ac:dyDescent="0.25">
@@ -60572,13 +60572,13 @@
         <v>13587.900709550519</v>
       </c>
       <c r="E127" s="18">
-        <v>-3617.19752695305</v>
+        <v>-3617.197526953049</v>
       </c>
       <c r="F127" s="18">
-        <v>-3375.1032904019944</v>
+        <v>-3375.103290401994</v>
       </c>
       <c r="G127" s="18">
-        <v>-1301.0748357081122</v>
+        <v>-1301.0748357081125</v>
       </c>
     </row>
     <row r="128" spans="2:7" x14ac:dyDescent="0.25">
@@ -60598,7 +60598,7 @@
         <v>-3356.19169752749</v>
       </c>
       <c r="G128" s="18">
-        <v>-1293.7845706480334</v>
+        <v>-1293.7845706480337</v>
       </c>
     </row>
     <row r="129" spans="2:7" x14ac:dyDescent="0.25">
@@ -60612,10 +60612,10 @@
         <v>15276.558196044107</v>
       </c>
       <c r="E129" s="18">
-        <v>-3097.997644831614</v>
+        <v>-3097.9976448316133</v>
       </c>
       <c r="F129" s="18">
-        <v>-2890.6527682873</v>
+        <v>-2890.6527682872998</v>
       </c>
       <c r="G129" s="18">
         <v>-1114.323104209545</v>
@@ -60649,7 +60649,7 @@
         <v>1</v>
       </c>
       <c r="D131" s="18">
-        <v>16663.240396056448</v>
+        <v>16663.24039605645</v>
       </c>
       <c r="E131" s="18">
         <v>-2631.40232041706</v>
@@ -60658,7 +60658,7 @@
         <v>-2455.2860505498015</v>
       </c>
       <c r="G131" s="18">
-        <v>-946.4927796194996</v>
+        <v>-946.4927796194999</v>
       </c>
     </row>
     <row r="132" spans="2:7" x14ac:dyDescent="0.25">
@@ -60692,13 +60692,13 @@
         <v>17312.418975260785</v>
       </c>
       <c r="E133" s="18">
-        <v>-2406.9025216643977</v>
+        <v>-2406.902521664397</v>
       </c>
       <c r="F133" s="18">
-        <v>-2245.8117257945937</v>
+        <v>-2245.8117257945933</v>
       </c>
       <c r="G133" s="18">
-        <v>-865.742133130844</v>
+        <v>-865.7421331308441</v>
       </c>
     </row>
     <row r="134" spans="2:7" x14ac:dyDescent="0.25">
@@ -60718,7 +60718,7 @@
         <v>-2085.2180703321987</v>
       </c>
       <c r="G134" s="18">
-        <v>-803.8345866297666</v>
+        <v>-803.8345866297667</v>
       </c>
     </row>
   </sheetData>

</xml_diff>